<commit_message>
Updated code after PK17 refresh
</commit_message>
<xml_diff>
--- a/Data/testDataCzechiaMK_ - Copy (3).xlsx
+++ b/Data/testDataCzechiaMK_ - Copy (3).xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27328"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5EB4817-6C69-42EC-88C1-F7C9C5B8DA10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF9F0ED1-5BF9-4A15-A912-0E1460950D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1367,7 +1367,7 @@
       </c>
       <c r="K2" s="20">
         <f t="shared" ref="K2:K14" ca="1" si="0">TODAY()-61</f>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="L2" s="16" t="s">
         <v>69</v>
@@ -1404,7 +1404,7 @@
       </c>
       <c r="W2" s="20">
         <f t="shared" ref="W2:W14" ca="1" si="1">K2</f>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="X2" s="19" t="s">
         <v>81</v>
@@ -1435,7 +1435,7 @@
       </c>
       <c r="AG2" s="27">
         <f t="shared" ref="AG2:AG14" ca="1" si="2">TODAY()+365</f>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AH2" s="28" t="s">
         <v>89</v>
@@ -1445,19 +1445,19 @@
       </c>
       <c r="AJ2" s="29">
         <f t="shared" ref="AJ2:AJ14" ca="1" si="3">K2</f>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AK2" s="27">
         <f t="shared" ref="AK2:AK14" ca="1" si="4">AG2</f>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AL2" s="30">
         <f t="shared" ref="AL2:AL14" ca="1" si="5">K2</f>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AM2" s="30">
         <f t="shared" ref="AM2:AM14" ca="1" si="6">K2</f>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AN2" s="28" t="s">
         <v>91</v>
@@ -1470,7 +1470,7 @@
       </c>
       <c r="AQ2" s="30">
         <f t="shared" ref="AQ2:AQ14" ca="1" si="7">TODAY()+20</f>
-        <v>45713</v>
+        <v>45729</v>
       </c>
       <c r="AR2" s="16" t="s">
         <v>69</v>
@@ -1593,7 +1593,7 @@
       </c>
       <c r="K3" s="20">
         <f t="shared" ca="1" si="0"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="L3" s="16" t="s">
         <v>69</v>
@@ -1630,7 +1630,7 @@
       </c>
       <c r="W3" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="X3" s="19" t="s">
         <v>81</v>
@@ -1661,7 +1661,7 @@
       </c>
       <c r="AG3" s="27">
         <f t="shared" ca="1" si="2"/>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AH3" s="28" t="s">
         <v>116</v>
@@ -1671,19 +1671,19 @@
       </c>
       <c r="AJ3" s="29">
         <f t="shared" ca="1" si="3"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AK3" s="27">
         <f t="shared" ca="1" si="4"/>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AL3" s="30">
         <f t="shared" ca="1" si="5"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AM3" s="30">
         <f t="shared" ca="1" si="6"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AN3" s="28" t="s">
         <v>91</v>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="AQ3" s="30">
         <f t="shared" ca="1" si="7"/>
-        <v>45713</v>
+        <v>45729</v>
       </c>
       <c r="AR3" s="16" t="s">
         <v>69</v>
@@ -1819,7 +1819,7 @@
       </c>
       <c r="K4" s="20">
         <f t="shared" ca="1" si="0"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="L4" s="16" t="s">
         <v>69</v>
@@ -1856,7 +1856,7 @@
       </c>
       <c r="W4" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="X4" s="19" t="s">
         <v>81</v>
@@ -1887,7 +1887,7 @@
       </c>
       <c r="AG4" s="27">
         <f t="shared" ca="1" si="2"/>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AH4" s="28" t="s">
         <v>116</v>
@@ -1897,19 +1897,19 @@
       </c>
       <c r="AJ4" s="29">
         <f t="shared" ca="1" si="3"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AK4" s="27">
         <f t="shared" ca="1" si="4"/>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AL4" s="30">
         <f t="shared" ca="1" si="5"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AM4" s="30">
         <f t="shared" ca="1" si="6"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AN4" s="28" t="s">
         <v>91</v>
@@ -1922,7 +1922,7 @@
       </c>
       <c r="AQ4" s="30">
         <f t="shared" ca="1" si="7"/>
-        <v>45713</v>
+        <v>45729</v>
       </c>
       <c r="AR4" s="16" t="s">
         <v>69</v>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="K5" s="20">
         <f t="shared" ca="1" si="0"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="L5" s="16" t="s">
         <v>69</v>
@@ -2082,7 +2082,7 @@
       </c>
       <c r="W5" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="X5" s="19" t="s">
         <v>81</v>
@@ -2113,7 +2113,7 @@
       </c>
       <c r="AG5" s="27">
         <f t="shared" ca="1" si="2"/>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AH5" s="28" t="s">
         <v>116</v>
@@ -2123,19 +2123,19 @@
       </c>
       <c r="AJ5" s="29">
         <f t="shared" ca="1" si="3"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AK5" s="27">
         <f t="shared" ca="1" si="4"/>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AL5" s="30">
         <f t="shared" ca="1" si="5"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AM5" s="30">
         <f t="shared" ca="1" si="6"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AN5" s="28" t="s">
         <v>91</v>
@@ -2148,7 +2148,7 @@
       </c>
       <c r="AQ5" s="30">
         <f t="shared" ca="1" si="7"/>
-        <v>45713</v>
+        <v>45729</v>
       </c>
       <c r="AR5" s="16" t="s">
         <v>69</v>
@@ -2271,7 +2271,7 @@
       </c>
       <c r="K6" s="20">
         <f t="shared" ca="1" si="0"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="L6" s="16" t="s">
         <v>69</v>
@@ -2308,7 +2308,7 @@
       </c>
       <c r="W6" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="X6" s="19" t="s">
         <v>81</v>
@@ -2339,7 +2339,7 @@
       </c>
       <c r="AG6" s="27">
         <f t="shared" ca="1" si="2"/>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AH6" s="28" t="s">
         <v>116</v>
@@ -2349,19 +2349,19 @@
       </c>
       <c r="AJ6" s="29">
         <f t="shared" ca="1" si="3"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AK6" s="27">
         <f t="shared" ca="1" si="4"/>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AL6" s="30">
         <f t="shared" ca="1" si="5"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AM6" s="30">
         <f t="shared" ca="1" si="6"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AN6" s="28" t="s">
         <v>91</v>
@@ -2374,7 +2374,7 @@
       </c>
       <c r="AQ6" s="30">
         <f t="shared" ca="1" si="7"/>
-        <v>45713</v>
+        <v>45729</v>
       </c>
       <c r="AR6" s="16" t="s">
         <v>69</v>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="K7" s="20">
         <f t="shared" ca="1" si="0"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="L7" s="16" t="s">
         <v>69</v>
@@ -2534,7 +2534,7 @@
       </c>
       <c r="W7" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="X7" s="19" t="s">
         <v>81</v>
@@ -2565,7 +2565,7 @@
       </c>
       <c r="AG7" s="27">
         <f t="shared" ca="1" si="2"/>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AH7" s="28" t="s">
         <v>116</v>
@@ -2575,19 +2575,19 @@
       </c>
       <c r="AJ7" s="29">
         <f t="shared" ca="1" si="3"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AK7" s="27">
         <f t="shared" ca="1" si="4"/>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AL7" s="30">
         <f t="shared" ca="1" si="5"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AM7" s="30">
         <f t="shared" ca="1" si="6"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AN7" s="28" t="s">
         <v>91</v>
@@ -2600,7 +2600,7 @@
       </c>
       <c r="AQ7" s="30">
         <f t="shared" ca="1" si="7"/>
-        <v>45713</v>
+        <v>45729</v>
       </c>
       <c r="AR7" s="16" t="s">
         <v>69</v>
@@ -2723,7 +2723,7 @@
       </c>
       <c r="K8" s="20">
         <f t="shared" ca="1" si="0"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="L8" s="16" t="s">
         <v>69</v>
@@ -2760,7 +2760,7 @@
       </c>
       <c r="W8" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="X8" s="19" t="s">
         <v>81</v>
@@ -2791,7 +2791,7 @@
       </c>
       <c r="AG8" s="27">
         <f t="shared" ca="1" si="2"/>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AH8" s="28" t="s">
         <v>116</v>
@@ -2801,19 +2801,19 @@
       </c>
       <c r="AJ8" s="29">
         <f t="shared" ca="1" si="3"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AK8" s="27">
         <f t="shared" ca="1" si="4"/>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AL8" s="30">
         <f t="shared" ca="1" si="5"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AM8" s="30">
         <f t="shared" ca="1" si="6"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AN8" s="28" t="s">
         <v>91</v>
@@ -2826,7 +2826,7 @@
       </c>
       <c r="AQ8" s="30">
         <f t="shared" ca="1" si="7"/>
-        <v>45713</v>
+        <v>45729</v>
       </c>
       <c r="AR8" s="16" t="s">
         <v>69</v>
@@ -2949,7 +2949,7 @@
       </c>
       <c r="K9" s="20">
         <f t="shared" ca="1" si="0"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="L9" s="16" t="s">
         <v>69</v>
@@ -2986,7 +2986,7 @@
       </c>
       <c r="W9" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="X9" s="19" t="s">
         <v>81</v>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="AG9" s="27">
         <f t="shared" ca="1" si="2"/>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AH9" s="28" t="s">
         <v>116</v>
@@ -3027,19 +3027,19 @@
       </c>
       <c r="AJ9" s="29">
         <f t="shared" ca="1" si="3"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AK9" s="27">
         <f t="shared" ca="1" si="4"/>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AL9" s="30">
         <f t="shared" ca="1" si="5"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AM9" s="30">
         <f t="shared" ca="1" si="6"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AN9" s="28" t="s">
         <v>91</v>
@@ -3052,7 +3052,7 @@
       </c>
       <c r="AQ9" s="30">
         <f t="shared" ca="1" si="7"/>
-        <v>45713</v>
+        <v>45729</v>
       </c>
       <c r="AR9" s="16" t="s">
         <v>69</v>
@@ -3175,7 +3175,7 @@
       </c>
       <c r="K10" s="20">
         <f t="shared" ca="1" si="0"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="L10" s="16" t="s">
         <v>69</v>
@@ -3212,7 +3212,7 @@
       </c>
       <c r="W10" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="X10" s="19" t="s">
         <v>81</v>
@@ -3243,7 +3243,7 @@
       </c>
       <c r="AG10" s="27">
         <f t="shared" ca="1" si="2"/>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AH10" s="28" t="s">
         <v>116</v>
@@ -3253,19 +3253,19 @@
       </c>
       <c r="AJ10" s="29">
         <f t="shared" ca="1" si="3"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AK10" s="27">
         <f t="shared" ca="1" si="4"/>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AL10" s="30">
         <f t="shared" ca="1" si="5"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AM10" s="30">
         <f t="shared" ca="1" si="6"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AN10" s="28" t="s">
         <v>91</v>
@@ -3278,7 +3278,7 @@
       </c>
       <c r="AQ10" s="30">
         <f t="shared" ca="1" si="7"/>
-        <v>45713</v>
+        <v>45729</v>
       </c>
       <c r="AR10" s="16" t="s">
         <v>69</v>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="K11" s="20">
         <f t="shared" ca="1" si="0"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="L11" s="16" t="s">
         <v>69</v>
@@ -3438,7 +3438,7 @@
       </c>
       <c r="W11" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="X11" s="19" t="s">
         <v>81</v>
@@ -3469,7 +3469,7 @@
       </c>
       <c r="AG11" s="27">
         <f t="shared" ca="1" si="2"/>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AH11" s="28" t="s">
         <v>116</v>
@@ -3479,19 +3479,19 @@
       </c>
       <c r="AJ11" s="29">
         <f t="shared" ca="1" si="3"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AK11" s="27">
         <f t="shared" ca="1" si="4"/>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AL11" s="30">
         <f t="shared" ca="1" si="5"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AM11" s="30">
         <f t="shared" ca="1" si="6"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AN11" s="28" t="s">
         <v>91</v>
@@ -3504,7 +3504,7 @@
       </c>
       <c r="AQ11" s="30">
         <f t="shared" ca="1" si="7"/>
-        <v>45713</v>
+        <v>45729</v>
       </c>
       <c r="AR11" s="16" t="s">
         <v>69</v>
@@ -3627,7 +3627,7 @@
       </c>
       <c r="K12" s="20">
         <f t="shared" ca="1" si="0"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="L12" s="16" t="s">
         <v>69</v>
@@ -3664,7 +3664,7 @@
       </c>
       <c r="W12" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="X12" s="19" t="s">
         <v>81</v>
@@ -3695,7 +3695,7 @@
       </c>
       <c r="AG12" s="27">
         <f t="shared" ca="1" si="2"/>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AH12" s="28" t="s">
         <v>116</v>
@@ -3705,19 +3705,19 @@
       </c>
       <c r="AJ12" s="29">
         <f t="shared" ca="1" si="3"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AK12" s="27">
         <f t="shared" ca="1" si="4"/>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AL12" s="30">
         <f t="shared" ca="1" si="5"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AM12" s="30">
         <f t="shared" ca="1" si="6"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AN12" s="28" t="s">
         <v>91</v>
@@ -3730,7 +3730,7 @@
       </c>
       <c r="AQ12" s="30">
         <f t="shared" ca="1" si="7"/>
-        <v>45713</v>
+        <v>45729</v>
       </c>
       <c r="AR12" s="16" t="s">
         <v>69</v>
@@ -3853,7 +3853,7 @@
       </c>
       <c r="K13" s="20">
         <f t="shared" ca="1" si="0"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="L13" s="16" t="s">
         <v>69</v>
@@ -3890,7 +3890,7 @@
       </c>
       <c r="W13" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="X13" s="19" t="s">
         <v>81</v>
@@ -3921,7 +3921,7 @@
       </c>
       <c r="AG13" s="27">
         <f t="shared" ca="1" si="2"/>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AH13" s="28" t="s">
         <v>116</v>
@@ -3931,19 +3931,19 @@
       </c>
       <c r="AJ13" s="29">
         <f t="shared" ca="1" si="3"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AK13" s="27">
         <f t="shared" ca="1" si="4"/>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AL13" s="30">
         <f t="shared" ca="1" si="5"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AM13" s="30">
         <f t="shared" ca="1" si="6"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AN13" s="28" t="s">
         <v>91</v>
@@ -3956,7 +3956,7 @@
       </c>
       <c r="AQ13" s="30">
         <f t="shared" ca="1" si="7"/>
-        <v>45713</v>
+        <v>45729</v>
       </c>
       <c r="AR13" s="16" t="s">
         <v>69</v>
@@ -4079,7 +4079,7 @@
       </c>
       <c r="K14" s="20">
         <f t="shared" ca="1" si="0"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="L14" s="16" t="s">
         <v>69</v>
@@ -4116,7 +4116,7 @@
       </c>
       <c r="W14" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="X14" s="19" t="s">
         <v>81</v>
@@ -4147,7 +4147,7 @@
       </c>
       <c r="AG14" s="27">
         <f t="shared" ca="1" si="2"/>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AH14" s="28" t="s">
         <v>116</v>
@@ -4157,19 +4157,19 @@
       </c>
       <c r="AJ14" s="29">
         <f t="shared" ca="1" si="3"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AK14" s="27">
         <f t="shared" ca="1" si="4"/>
-        <v>46058</v>
+        <v>46074</v>
       </c>
       <c r="AL14" s="30">
         <f t="shared" ca="1" si="5"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AM14" s="30">
         <f t="shared" ca="1" si="6"/>
-        <v>45632</v>
+        <v>45648</v>
       </c>
       <c r="AN14" s="28" t="s">
         <v>91</v>
@@ -4182,7 +4182,7 @@
       </c>
       <c r="AQ14" s="30">
         <f t="shared" ca="1" si="7"/>
-        <v>45713</v>
+        <v>45729</v>
       </c>
       <c r="AR14" s="16" t="s">
         <v>69</v>

</xml_diff>